<commit_message>
fix: map function list change status input
</commit_message>
<xml_diff>
--- a/tests/fixtures/功能清单-录入模板.xlsx
+++ b/tests/fixtures/功能清单-录入模板.xlsx
@@ -558,12 +558,12 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>功能过程类型</t>
+          <t>功能过程描述</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>功能过程描述</t>
+          <t>变更状态</t>
         </is>
       </c>
     </row>
@@ -605,12 +605,12 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>EI</t>
+          <t>接收用户的注册请求数据</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>接收用户的注册请求数据</t>
+          <t>新增</t>
         </is>
       </c>
     </row>
@@ -652,12 +652,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>R</t>
+          <t>校验用户名是否已存在</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>校验用户名是否已存在</t>
+          <t>新增</t>
         </is>
       </c>
     </row>
@@ -699,12 +699,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>将用户信息写入数据库</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>将用户信息写入数据库</t>
+          <t>新增</t>
         </is>
       </c>
     </row>
@@ -746,12 +746,12 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>接收用户输入的查询条件</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>接收用户输入的查询条件</t>
+          <t>新增</t>
         </is>
       </c>
     </row>
@@ -793,12 +793,12 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>返回符合条件的用户列表</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>返回符合条件的用户列表</t>
+          <t>新增</t>
         </is>
       </c>
     </row>
@@ -840,12 +840,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>接收角色名称和权限列表</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>接收角色名称和权限列表</t>
+          <t>新增</t>
         </is>
       </c>
     </row>
@@ -887,12 +887,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>将角色信息写入数据库</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>将角色信息写入数据库</t>
+          <t>新增</t>
         </is>
       </c>
     </row>

</xml_diff>